<commit_message>
feat(backend): updated base template
</commit_message>
<xml_diff>
--- a/backend/templates/base_template.xlsx
+++ b/backend/templates/base_template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasmckenzie/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9AC422-3AE1-F94E-91A8-87AB1D9CA51C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D457ED-154F-6049-A60D-7FC85F7A5899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="4" xr2:uid="{98C021A7-547A-C84F-B88C-65745982F461}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="2" xr2:uid="{98C021A7-547A-C84F-B88C-65745982F461}"/>
   </bookViews>
   <sheets>
     <sheet name="Roll Up Template" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="107">
   <si>
     <t>Production Month:</t>
   </si>
@@ -352,6 +352,12 @@
   </si>
   <si>
     <t>Fluid in Disposal Tanks</t>
+  </si>
+  <si>
+    <t>Well Template</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -2201,28 +2207,28 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3131,56 +3137,150 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -3242,13 +3342,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -3257,6 +3350,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -3321,8 +3421,33 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
@@ -10286,9 +10411,8 @@
       <c r="AD1" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="AE1" s="50" t="str">
-        <f ca="1">RIGHT(CELL("filename",A1),LEN(CELL("filename",A1))-FIND("]",CELL("filename",A1),1))</f>
-        <v>Well Template</v>
+      <c r="AE1" s="50" t="s">
+        <v>105</v>
       </c>
       <c r="AF1" s="45"/>
       <c r="AG1" s="45"/>
@@ -10807,40 +10931,33 @@
         <v>1</v>
       </c>
       <c r="B7" s="160"/>
-      <c r="C7" s="86" t="str">
-        <f t="shared" ref="C7:C37" si="0">IF(ISBLANK(B7),"",24-B7)</f>
-        <v/>
+      <c r="C7" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D7" s="161"/>
       <c r="E7" s="162"/>
       <c r="F7" s="162"/>
-      <c r="G7" s="87" t="str">
-        <f>IF(ISBLANK(B7),"",E40+H7-(M7+Q7+R7+(#REF!-U7)+V7))</f>
-        <v/>
+      <c r="G7" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H7" s="163"/>
-      <c r="I7" s="88" t="str">
-        <f t="shared" ref="I7:I37" si="1">IF(ISBLANK(H7),"",+H7*(1-E7))</f>
-        <v/>
-      </c>
-      <c r="J7" s="89" t="str">
-        <f t="shared" ref="J7:J37" si="2">IF(ISBLANK(H7),"",+H7*(F7))</f>
-        <v/>
-      </c>
-      <c r="K7" s="88" t="str">
-        <f t="shared" ref="K7:K37" si="3">IF(ISBLANK(H7),"",+H7*(E7-F7))</f>
-        <v/>
+      <c r="I7" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J7" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K7" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L7" s="184"/>
       <c r="M7" s="165"/>
       <c r="N7" s="164"/>
-      <c r="O7" s="90" t="str">
-        <f t="shared" ref="O7:O37" si="4">IF(ISBLANK(H7),"",+M7*(1-N7))</f>
-        <v/>
-      </c>
-      <c r="P7" s="90" t="str">
-        <f t="shared" ref="P7:P37" si="5">IF(ISBLANK(H7),"",+M7*N7)</f>
-        <v/>
+      <c r="O7" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P7" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q7" s="237"/>
       <c r="R7" s="244"/>
@@ -10854,17 +10971,11 @@
       <c r="Z7" s="166"/>
       <c r="AA7" s="168"/>
       <c r="AB7" s="168"/>
-      <c r="AC7" s="93" t="e">
-        <f t="shared" ref="AC7:AC38" si="6">+H7/($I$3*AB7/100)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC7" s="93"/>
       <c r="AD7" s="168"/>
       <c r="AE7" s="176"/>
       <c r="AF7" s="189"/>
-      <c r="AG7" s="127" t="str">
-        <f>IF(AH7+AN7=G7,G7,"REDO")</f>
-        <v>REDO</v>
-      </c>
+      <c r="AG7" s="127"/>
       <c r="AH7" s="186"/>
       <c r="AI7" s="173"/>
       <c r="AJ7" s="174"/>
@@ -10900,44 +11011,36 @@
     </row>
     <row r="8" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="94">
-        <f t="shared" ref="A8:A13" si="7">+A7+1</f>
         <v>2</v>
       </c>
       <c r="B8" s="160"/>
-      <c r="C8" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C8" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D8" s="198"/>
       <c r="E8" s="162"/>
       <c r="F8" s="162"/>
-      <c r="G8" s="87" t="str">
-        <f>IF(ISBLANK(B8),"",G7+H8-(M8+Q8+R8+(T7-U8)+V8))</f>
-        <v/>
+      <c r="G8" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H8" s="163"/>
-      <c r="I8" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J8" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K8" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I8" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J8" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K8" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L8" s="187"/>
       <c r="M8" s="188"/>
       <c r="N8" s="171"/>
-      <c r="O8" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P8" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O8" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P8" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q8" s="243"/>
       <c r="R8" s="244"/>
@@ -10950,17 +11053,11 @@
       <c r="Z8" s="166"/>
       <c r="AA8" s="168"/>
       <c r="AB8" s="168"/>
-      <c r="AC8" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC8" s="93"/>
       <c r="AD8" s="168"/>
       <c r="AE8" s="175"/>
       <c r="AF8" s="189"/>
-      <c r="AG8" s="127" t="str">
-        <f t="shared" ref="AG8:AG37" si="8">IF(AH8+AN8=G8,G8,"REDO")</f>
-        <v>REDO</v>
-      </c>
+      <c r="AG8" s="127"/>
       <c r="AH8" s="186"/>
       <c r="AI8" s="173"/>
       <c r="AJ8" s="174"/>
@@ -10996,44 +11093,36 @@
     </row>
     <row r="9" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="94">
-        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="B9" s="160"/>
-      <c r="C9" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C9" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D9" s="183"/>
       <c r="E9" s="162"/>
       <c r="F9" s="162"/>
-      <c r="G9" s="87" t="str">
-        <f t="shared" ref="G9:G37" si="9">IF(ISBLANK(B9),"",G8+H9-(M9+Q9+R9+(T9-U9)+V9))</f>
-        <v/>
+      <c r="G9" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H9" s="163"/>
-      <c r="I9" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J9" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K9" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I9" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J9" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K9" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L9" s="187"/>
       <c r="M9" s="188"/>
       <c r="N9" s="171"/>
-      <c r="O9" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P9" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O9" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P9" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q9" s="243"/>
       <c r="R9" s="244"/>
@@ -11047,17 +11136,11 @@
       <c r="Z9" s="166"/>
       <c r="AA9" s="168"/>
       <c r="AB9" s="168"/>
-      <c r="AC9" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC9" s="93"/>
       <c r="AD9" s="168"/>
       <c r="AE9" s="169"/>
       <c r="AF9" s="189"/>
-      <c r="AG9" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG9" s="128"/>
       <c r="AH9" s="186"/>
       <c r="AI9" s="173"/>
       <c r="AJ9" s="174"/>
@@ -11093,44 +11176,36 @@
     </row>
     <row r="10" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="94">
-        <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="B10" s="160"/>
-      <c r="C10" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C10" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D10" s="198"/>
       <c r="E10" s="162"/>
       <c r="F10" s="162"/>
-      <c r="G10" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G10" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H10" s="163"/>
-      <c r="I10" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J10" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K10" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I10" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J10" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K10" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L10" s="187"/>
       <c r="M10" s="188"/>
       <c r="N10" s="171"/>
-      <c r="O10" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P10" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O10" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P10" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q10" s="243"/>
       <c r="R10" s="244"/>
@@ -11144,17 +11219,11 @@
       <c r="Z10" s="166"/>
       <c r="AA10" s="168"/>
       <c r="AB10" s="168"/>
-      <c r="AC10" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC10" s="93"/>
       <c r="AD10" s="168"/>
       <c r="AE10" s="169"/>
       <c r="AF10" s="189"/>
-      <c r="AG10" s="127" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG10" s="127"/>
       <c r="AH10" s="186"/>
       <c r="AI10" s="173"/>
       <c r="AJ10" s="174"/>
@@ -11190,44 +11259,36 @@
     </row>
     <row r="11" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="94">
-        <f t="shared" si="7"/>
         <v>5</v>
       </c>
       <c r="B11" s="160"/>
-      <c r="C11" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C11" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D11" s="183"/>
       <c r="E11" s="162"/>
       <c r="F11" s="162"/>
-      <c r="G11" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G11" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H11" s="163"/>
-      <c r="I11" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J11" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K11" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I11" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J11" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K11" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L11" s="187"/>
       <c r="M11" s="188"/>
       <c r="N11" s="171"/>
-      <c r="O11" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P11" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O11" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P11" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q11" s="243"/>
       <c r="R11" s="244"/>
@@ -11241,17 +11302,11 @@
       <c r="Z11" s="166"/>
       <c r="AA11" s="168"/>
       <c r="AB11" s="168"/>
-      <c r="AC11" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC11" s="93"/>
       <c r="AD11" s="168"/>
       <c r="AE11" s="169"/>
       <c r="AF11" s="189"/>
-      <c r="AG11" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG11" s="128"/>
       <c r="AH11" s="186"/>
       <c r="AI11" s="173"/>
       <c r="AJ11" s="174"/>
@@ -11287,44 +11342,36 @@
     </row>
     <row r="12" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="94">
-        <f t="shared" si="7"/>
         <v>6</v>
       </c>
       <c r="B12" s="160"/>
-      <c r="C12" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C12" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D12" s="198"/>
       <c r="E12" s="162"/>
       <c r="F12" s="162"/>
-      <c r="G12" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G12" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H12" s="163"/>
-      <c r="I12" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J12" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K12" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I12" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J12" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K12" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L12" s="187"/>
       <c r="M12" s="188"/>
       <c r="N12" s="171"/>
-      <c r="O12" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P12" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O12" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P12" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q12" s="243"/>
       <c r="R12" s="244"/>
@@ -11338,17 +11385,11 @@
       <c r="Z12" s="166"/>
       <c r="AA12" s="168"/>
       <c r="AB12" s="168"/>
-      <c r="AC12" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC12" s="93"/>
       <c r="AD12" s="265"/>
       <c r="AE12" s="169"/>
       <c r="AF12" s="189"/>
-      <c r="AG12" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG12" s="128"/>
       <c r="AH12" s="186"/>
       <c r="AI12" s="173"/>
       <c r="AJ12" s="174"/>
@@ -11384,44 +11425,36 @@
     </row>
     <row r="13" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="94">
-        <f t="shared" si="7"/>
         <v>7</v>
       </c>
       <c r="B13" s="160"/>
-      <c r="C13" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C13" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D13" s="183"/>
       <c r="E13" s="162"/>
       <c r="F13" s="162"/>
-      <c r="G13" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G13" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H13" s="163"/>
-      <c r="I13" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J13" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K13" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I13" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J13" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K13" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L13" s="187"/>
       <c r="M13" s="188"/>
       <c r="N13" s="171"/>
-      <c r="O13" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P13" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O13" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P13" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q13" s="243"/>
       <c r="R13" s="244"/>
@@ -11435,17 +11468,11 @@
       <c r="Z13" s="166"/>
       <c r="AA13" s="168"/>
       <c r="AB13" s="168"/>
-      <c r="AC13" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC13" s="93"/>
       <c r="AD13" s="168"/>
       <c r="AE13" s="169"/>
       <c r="AF13" s="189"/>
-      <c r="AG13" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG13" s="128"/>
       <c r="AH13" s="186"/>
       <c r="AI13" s="173"/>
       <c r="AJ13" s="174"/>
@@ -11484,40 +11511,33 @@
         <v>8</v>
       </c>
       <c r="B14" s="160"/>
-      <c r="C14" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C14" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D14" s="198"/>
       <c r="E14" s="162"/>
       <c r="F14" s="162"/>
-      <c r="G14" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G14" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H14" s="163"/>
-      <c r="I14" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J14" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K14" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I14" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J14" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K14" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L14" s="187"/>
       <c r="M14" s="188"/>
       <c r="N14" s="177"/>
-      <c r="O14" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P14" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O14" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P14" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q14" s="243"/>
       <c r="R14" s="244"/>
@@ -11531,17 +11551,11 @@
       <c r="Z14" s="166"/>
       <c r="AA14" s="168"/>
       <c r="AB14" s="168"/>
-      <c r="AC14" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC14" s="93"/>
       <c r="AD14" s="168"/>
       <c r="AE14" s="169"/>
       <c r="AF14" s="189"/>
-      <c r="AG14" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG14" s="128"/>
       <c r="AH14" s="186"/>
       <c r="AI14" s="173"/>
       <c r="AJ14" s="174"/>
@@ -11577,44 +11591,36 @@
     </row>
     <row r="15" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="94">
-        <f t="shared" ref="A15:A37" si="10">+A14+1</f>
         <v>9</v>
       </c>
       <c r="B15" s="160"/>
-      <c r="C15" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C15" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D15" s="183"/>
       <c r="E15" s="162"/>
       <c r="F15" s="162"/>
-      <c r="G15" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G15" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H15" s="163"/>
-      <c r="I15" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J15" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K15" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I15" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J15" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K15" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L15" s="187"/>
       <c r="M15" s="255"/>
       <c r="N15" s="257"/>
-      <c r="O15" s="256" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P15" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O15" s="256" t="s">
+        <v>106</v>
+      </c>
+      <c r="P15" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q15" s="243"/>
       <c r="R15" s="244"/>
@@ -11628,17 +11634,11 @@
       <c r="Z15" s="166"/>
       <c r="AA15" s="168"/>
       <c r="AB15" s="168"/>
-      <c r="AC15" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC15" s="93"/>
       <c r="AD15" s="168"/>
       <c r="AE15" s="169"/>
       <c r="AF15" s="189"/>
-      <c r="AG15" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG15" s="128"/>
       <c r="AH15" s="186"/>
       <c r="AI15" s="173"/>
       <c r="AJ15" s="174"/>
@@ -11674,44 +11674,36 @@
     </row>
     <row r="16" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="94">
-        <f t="shared" si="10"/>
         <v>10</v>
       </c>
       <c r="B16" s="160"/>
-      <c r="C16" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C16" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D16" s="198"/>
       <c r="E16" s="162"/>
       <c r="F16" s="162"/>
-      <c r="G16" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G16" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H16" s="172"/>
-      <c r="I16" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J16" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K16" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I16" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J16" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K16" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L16" s="187"/>
       <c r="M16" s="188"/>
       <c r="N16" s="164"/>
-      <c r="O16" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P16" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O16" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P16" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q16" s="243"/>
       <c r="R16" s="244"/>
@@ -11725,17 +11717,11 @@
       <c r="Z16" s="166"/>
       <c r="AA16" s="168"/>
       <c r="AB16" s="168"/>
-      <c r="AC16" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC16" s="93"/>
       <c r="AD16" s="168"/>
       <c r="AE16" s="169"/>
       <c r="AF16" s="189"/>
-      <c r="AG16" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG16" s="128"/>
       <c r="AH16" s="186"/>
       <c r="AI16" s="173"/>
       <c r="AJ16" s="174"/>
@@ -11771,44 +11757,36 @@
     </row>
     <row r="17" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="94">
-        <f t="shared" si="10"/>
         <v>11</v>
       </c>
       <c r="B17" s="160"/>
-      <c r="C17" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C17" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D17" s="183"/>
       <c r="E17" s="162"/>
       <c r="F17" s="162"/>
-      <c r="G17" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G17" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H17" s="172"/>
-      <c r="I17" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J17" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K17" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I17" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J17" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K17" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L17" s="187"/>
       <c r="M17" s="188"/>
       <c r="N17" s="171"/>
-      <c r="O17" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P17" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O17" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P17" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q17" s="243"/>
       <c r="R17" s="244"/>
@@ -11822,17 +11800,11 @@
       <c r="Z17" s="166"/>
       <c r="AA17" s="168"/>
       <c r="AB17" s="168"/>
-      <c r="AC17" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC17" s="93"/>
       <c r="AD17" s="168"/>
       <c r="AE17" s="169"/>
       <c r="AF17" s="266"/>
-      <c r="AG17" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG17" s="128"/>
       <c r="AH17" s="186"/>
       <c r="AI17" s="173"/>
       <c r="AJ17" s="174"/>
@@ -11868,44 +11840,36 @@
     </row>
     <row r="18" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="94">
-        <f t="shared" si="10"/>
         <v>12</v>
       </c>
       <c r="B18" s="160"/>
-      <c r="C18" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C18" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D18" s="198"/>
       <c r="E18" s="162"/>
       <c r="F18" s="162"/>
-      <c r="G18" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G18" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H18" s="172"/>
-      <c r="I18" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J18" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K18" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I18" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J18" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K18" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L18" s="187"/>
       <c r="M18" s="188"/>
       <c r="N18" s="171"/>
-      <c r="O18" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P18" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O18" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P18" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q18" s="243"/>
       <c r="R18" s="244"/>
@@ -11919,17 +11883,11 @@
       <c r="Z18" s="166"/>
       <c r="AA18" s="168"/>
       <c r="AB18" s="168"/>
-      <c r="AC18" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC18" s="93"/>
       <c r="AD18" s="168"/>
       <c r="AE18" s="169"/>
       <c r="AF18" s="266"/>
-      <c r="AG18" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG18" s="128"/>
       <c r="AH18" s="186"/>
       <c r="AI18" s="173"/>
       <c r="AJ18" s="174"/>
@@ -11965,44 +11923,36 @@
     </row>
     <row r="19" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="94">
-        <f t="shared" si="10"/>
         <v>13</v>
       </c>
       <c r="B19" s="160"/>
-      <c r="C19" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C19" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D19" s="183"/>
       <c r="E19" s="162"/>
       <c r="F19" s="162"/>
-      <c r="G19" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G19" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H19" s="172"/>
-      <c r="I19" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J19" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K19" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I19" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J19" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K19" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L19" s="187"/>
       <c r="M19" s="188"/>
       <c r="N19" s="171"/>
-      <c r="O19" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P19" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O19" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P19" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q19" s="243"/>
       <c r="R19" s="244"/>
@@ -12016,17 +11966,11 @@
       <c r="Z19" s="166"/>
       <c r="AA19" s="168"/>
       <c r="AB19" s="168"/>
-      <c r="AC19" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC19" s="93"/>
       <c r="AD19" s="168"/>
       <c r="AE19" s="169"/>
       <c r="AF19" s="267"/>
-      <c r="AG19" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG19" s="128"/>
       <c r="AH19" s="186"/>
       <c r="AI19" s="173"/>
       <c r="AJ19" s="174"/>
@@ -12062,44 +12006,36 @@
     </row>
     <row r="20" spans="1:65" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="94">
-        <f t="shared" si="10"/>
         <v>14</v>
       </c>
       <c r="B20" s="160"/>
-      <c r="C20" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C20" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D20" s="198"/>
       <c r="E20" s="162"/>
       <c r="F20" s="162"/>
-      <c r="G20" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G20" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H20" s="172"/>
-      <c r="I20" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J20" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K20" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I20" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J20" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K20" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L20" s="187"/>
       <c r="M20" s="188"/>
       <c r="N20" s="171"/>
-      <c r="O20" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P20" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O20" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P20" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q20" s="243"/>
       <c r="R20" s="244"/>
@@ -12113,17 +12049,11 @@
       <c r="Z20" s="166"/>
       <c r="AA20" s="168"/>
       <c r="AB20" s="168"/>
-      <c r="AC20" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC20" s="93"/>
       <c r="AD20" s="168"/>
       <c r="AE20" s="169"/>
       <c r="AF20" s="266"/>
-      <c r="AG20" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG20" s="128"/>
       <c r="AH20" s="186"/>
       <c r="AI20" s="173"/>
       <c r="AJ20" s="174"/>
@@ -12159,44 +12089,36 @@
     </row>
     <row r="21" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="94">
-        <f t="shared" si="10"/>
         <v>15</v>
       </c>
       <c r="B21" s="160"/>
-      <c r="C21" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C21" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D21" s="183"/>
       <c r="E21" s="162"/>
       <c r="F21" s="162"/>
-      <c r="G21" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G21" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H21" s="172"/>
-      <c r="I21" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J21" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K21" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I21" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J21" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K21" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L21" s="187"/>
       <c r="M21" s="188"/>
       <c r="N21" s="171"/>
-      <c r="O21" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P21" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O21" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P21" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q21" s="243"/>
       <c r="R21" s="244"/>
@@ -12210,17 +12132,11 @@
       <c r="Z21" s="166"/>
       <c r="AA21" s="168"/>
       <c r="AB21" s="168"/>
-      <c r="AC21" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC21" s="93"/>
       <c r="AD21" s="168"/>
       <c r="AE21" s="169"/>
       <c r="AF21" s="266"/>
-      <c r="AG21" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG21" s="128"/>
       <c r="AH21" s="186"/>
       <c r="AI21" s="173"/>
       <c r="AJ21" s="174"/>
@@ -12256,44 +12172,36 @@
     </row>
     <row r="22" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="94">
-        <f t="shared" si="10"/>
         <v>16</v>
       </c>
       <c r="B22" s="160"/>
-      <c r="C22" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C22" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D22" s="198"/>
       <c r="E22" s="162"/>
       <c r="F22" s="162"/>
-      <c r="G22" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G22" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H22" s="172"/>
-      <c r="I22" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J22" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K22" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I22" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J22" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K22" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L22" s="187"/>
       <c r="M22" s="188"/>
       <c r="N22" s="171"/>
-      <c r="O22" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P22" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O22" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P22" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q22" s="243"/>
       <c r="R22" s="244"/>
@@ -12307,17 +12215,11 @@
       <c r="Z22" s="166"/>
       <c r="AA22" s="168"/>
       <c r="AB22" s="168"/>
-      <c r="AC22" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC22" s="93"/>
       <c r="AD22" s="168"/>
       <c r="AE22" s="169"/>
       <c r="AF22" s="266"/>
-      <c r="AG22" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG22" s="128"/>
       <c r="AH22" s="186"/>
       <c r="AI22" s="173"/>
       <c r="AJ22" s="174"/>
@@ -12353,44 +12255,36 @@
     </row>
     <row r="23" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="94">
-        <f t="shared" si="10"/>
         <v>17</v>
       </c>
       <c r="B23" s="160"/>
-      <c r="C23" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C23" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D23" s="183"/>
       <c r="E23" s="162"/>
       <c r="F23" s="162"/>
-      <c r="G23" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G23" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H23" s="172"/>
-      <c r="I23" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J23" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K23" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I23" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J23" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K23" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L23" s="187"/>
       <c r="M23" s="188"/>
       <c r="N23" s="171"/>
-      <c r="O23" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P23" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O23" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P23" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q23" s="243"/>
       <c r="R23" s="244"/>
@@ -12404,17 +12298,11 @@
       <c r="Z23" s="166"/>
       <c r="AA23" s="168"/>
       <c r="AB23" s="168"/>
-      <c r="AC23" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC23" s="93"/>
       <c r="AD23" s="168"/>
       <c r="AE23" s="169"/>
       <c r="AF23" s="268"/>
-      <c r="AG23" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG23" s="128"/>
       <c r="AH23" s="186"/>
       <c r="AI23" s="173"/>
       <c r="AJ23" s="174"/>
@@ -12450,44 +12338,36 @@
     </row>
     <row r="24" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="94">
-        <f t="shared" si="10"/>
         <v>18</v>
       </c>
       <c r="B24" s="160"/>
-      <c r="C24" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C24" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D24" s="198"/>
       <c r="E24" s="162"/>
       <c r="F24" s="162"/>
-      <c r="G24" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G24" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H24" s="172"/>
-      <c r="I24" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J24" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K24" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I24" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J24" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K24" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L24" s="187"/>
       <c r="M24" s="188"/>
       <c r="N24" s="171"/>
-      <c r="O24" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P24" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O24" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P24" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q24" s="243"/>
       <c r="R24" s="244"/>
@@ -12501,17 +12381,11 @@
       <c r="Z24" s="166"/>
       <c r="AA24" s="168"/>
       <c r="AB24" s="168"/>
-      <c r="AC24" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC24" s="93"/>
       <c r="AD24" s="168"/>
       <c r="AE24" s="169"/>
       <c r="AF24" s="170"/>
-      <c r="AG24" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG24" s="128"/>
       <c r="AH24" s="186"/>
       <c r="AI24" s="173"/>
       <c r="AJ24" s="174"/>
@@ -12547,44 +12421,36 @@
     </row>
     <row r="25" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="94">
-        <f t="shared" si="10"/>
         <v>19</v>
       </c>
       <c r="B25" s="160"/>
-      <c r="C25" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C25" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D25" s="183"/>
       <c r="E25" s="162"/>
       <c r="F25" s="162"/>
-      <c r="G25" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G25" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H25" s="172"/>
-      <c r="I25" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J25" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K25" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I25" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J25" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K25" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L25" s="187"/>
       <c r="M25" s="188"/>
       <c r="N25" s="171"/>
-      <c r="O25" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P25" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O25" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P25" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q25" s="243"/>
       <c r="R25" s="244"/>
@@ -12600,17 +12466,11 @@
       <c r="Z25" s="166"/>
       <c r="AA25" s="168"/>
       <c r="AB25" s="168"/>
-      <c r="AC25" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC25" s="93"/>
       <c r="AD25" s="168"/>
       <c r="AE25" s="169"/>
       <c r="AF25" s="170"/>
-      <c r="AG25" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG25" s="128"/>
       <c r="AH25" s="186"/>
       <c r="AI25" s="173"/>
       <c r="AJ25" s="174"/>
@@ -12646,44 +12506,36 @@
     </row>
     <row r="26" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="94">
-        <f t="shared" si="10"/>
         <v>20</v>
       </c>
       <c r="B26" s="160"/>
-      <c r="C26" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C26" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D26" s="198"/>
       <c r="E26" s="162"/>
       <c r="F26" s="162"/>
-      <c r="G26" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G26" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H26" s="172"/>
-      <c r="I26" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J26" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K26" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I26" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J26" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K26" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L26" s="187"/>
       <c r="M26" s="188"/>
       <c r="N26" s="171"/>
-      <c r="O26" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P26" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O26" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P26" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q26" s="243"/>
       <c r="R26" s="244"/>
@@ -12697,17 +12549,11 @@
       <c r="Z26" s="166"/>
       <c r="AA26" s="168"/>
       <c r="AB26" s="168"/>
-      <c r="AC26" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC26" s="93"/>
       <c r="AD26" s="168"/>
       <c r="AE26" s="169"/>
       <c r="AF26" s="170"/>
-      <c r="AG26" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG26" s="128"/>
       <c r="AH26" s="186"/>
       <c r="AI26" s="173"/>
       <c r="AJ26" s="174"/>
@@ -12743,44 +12589,36 @@
     </row>
     <row r="27" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="94">
-        <f t="shared" si="10"/>
         <v>21</v>
       </c>
       <c r="B27" s="160"/>
-      <c r="C27" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C27" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D27" s="183"/>
       <c r="E27" s="162"/>
       <c r="F27" s="162"/>
-      <c r="G27" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G27" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H27" s="172"/>
-      <c r="I27" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J27" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K27" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I27" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J27" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K27" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L27" s="187"/>
       <c r="M27" s="188"/>
       <c r="N27" s="171"/>
-      <c r="O27" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P27" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O27" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P27" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q27" s="243"/>
       <c r="R27" s="244"/>
@@ -12794,17 +12632,11 @@
       <c r="Z27" s="166"/>
       <c r="AA27" s="168"/>
       <c r="AB27" s="168"/>
-      <c r="AC27" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC27" s="93"/>
       <c r="AD27" s="168"/>
       <c r="AE27" s="169"/>
       <c r="AF27" s="170"/>
-      <c r="AG27" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG27" s="128"/>
       <c r="AH27" s="186"/>
       <c r="AI27" s="173"/>
       <c r="AJ27" s="174"/>
@@ -12840,44 +12672,36 @@
     </row>
     <row r="28" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="94">
-        <f t="shared" si="10"/>
         <v>22</v>
       </c>
       <c r="B28" s="160"/>
-      <c r="C28" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C28" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D28" s="183"/>
       <c r="E28" s="162"/>
       <c r="F28" s="162"/>
-      <c r="G28" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G28" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H28" s="172"/>
-      <c r="I28" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J28" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K28" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I28" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J28" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K28" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L28" s="187"/>
       <c r="M28" s="188"/>
       <c r="N28" s="171"/>
-      <c r="O28" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P28" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O28" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P28" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q28" s="243"/>
       <c r="R28" s="244"/>
@@ -12891,17 +12715,11 @@
       <c r="Z28" s="166"/>
       <c r="AA28" s="168"/>
       <c r="AB28" s="168"/>
-      <c r="AC28" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC28" s="93"/>
       <c r="AD28" s="168"/>
       <c r="AE28" s="176"/>
       <c r="AF28" s="170"/>
-      <c r="AG28" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG28" s="128"/>
       <c r="AH28" s="186"/>
       <c r="AI28" s="173"/>
       <c r="AJ28" s="174"/>
@@ -12937,44 +12755,36 @@
     </row>
     <row r="29" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="94">
-        <f t="shared" si="10"/>
         <v>23</v>
       </c>
       <c r="B29" s="160"/>
-      <c r="C29" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C29" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D29" s="183"/>
       <c r="E29" s="162"/>
       <c r="F29" s="162"/>
-      <c r="G29" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G29" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H29" s="172"/>
-      <c r="I29" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J29" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K29" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I29" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J29" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K29" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L29" s="187"/>
       <c r="M29" s="188"/>
       <c r="N29" s="171"/>
-      <c r="O29" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P29" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O29" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P29" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q29" s="243"/>
       <c r="R29" s="244"/>
@@ -12988,17 +12798,11 @@
       <c r="Z29" s="166"/>
       <c r="AA29" s="168"/>
       <c r="AB29" s="168"/>
-      <c r="AC29" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC29" s="93"/>
       <c r="AD29" s="168"/>
       <c r="AE29" s="176"/>
       <c r="AF29" s="170"/>
-      <c r="AG29" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG29" s="128"/>
       <c r="AH29" s="186"/>
       <c r="AI29" s="173"/>
       <c r="AJ29" s="174"/>
@@ -13034,44 +12838,36 @@
     </row>
     <row r="30" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="94">
-        <f t="shared" si="10"/>
         <v>24</v>
       </c>
       <c r="B30" s="160"/>
-      <c r="C30" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C30" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D30" s="183"/>
       <c r="E30" s="162"/>
       <c r="F30" s="162"/>
-      <c r="G30" s="87" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G30" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H30" s="172"/>
-      <c r="I30" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J30" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K30" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I30" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J30" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K30" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L30" s="187"/>
       <c r="M30" s="188"/>
       <c r="N30" s="171"/>
-      <c r="O30" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P30" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O30" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P30" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q30" s="243"/>
       <c r="R30" s="244"/>
@@ -13085,17 +12881,11 @@
       <c r="Z30" s="166"/>
       <c r="AA30" s="168"/>
       <c r="AB30" s="168"/>
-      <c r="AC30" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC30" s="93"/>
       <c r="AD30" s="168"/>
       <c r="AE30" s="176"/>
       <c r="AF30" s="170"/>
-      <c r="AG30" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG30" s="128"/>
       <c r="AH30" s="186"/>
       <c r="AI30" s="173"/>
       <c r="AJ30" s="174"/>
@@ -13131,44 +12921,36 @@
     </row>
     <row r="31" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="94">
-        <f t="shared" si="10"/>
         <v>25</v>
       </c>
       <c r="B31" s="160"/>
-      <c r="C31" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C31" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D31" s="183"/>
       <c r="E31" s="162"/>
       <c r="F31" s="162"/>
-      <c r="G31" s="87" t="str">
-        <f t="shared" ref="G31:G36" si="11">IF(ISBLANK(B31),"",G30+H31-(M31+Q31+R31+(T31-U31)+V31))</f>
-        <v/>
+      <c r="G31" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H31" s="172"/>
-      <c r="I31" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J31" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K31" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I31" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J31" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K31" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L31" s="187"/>
       <c r="M31" s="188"/>
       <c r="N31" s="171"/>
-      <c r="O31" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P31" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O31" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P31" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q31" s="243"/>
       <c r="R31" s="244"/>
@@ -13182,17 +12964,11 @@
       <c r="Z31" s="166"/>
       <c r="AA31" s="168"/>
       <c r="AB31" s="168"/>
-      <c r="AC31" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC31" s="93"/>
       <c r="AD31" s="168"/>
       <c r="AE31" s="176"/>
       <c r="AF31" s="189"/>
-      <c r="AG31" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG31" s="128"/>
       <c r="AH31" s="186"/>
       <c r="AI31" s="173"/>
       <c r="AJ31" s="174"/>
@@ -13228,44 +13004,36 @@
     </row>
     <row r="32" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="94">
-        <f t="shared" si="10"/>
         <v>26</v>
       </c>
       <c r="B32" s="160"/>
-      <c r="C32" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C32" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D32" s="183"/>
       <c r="E32" s="162"/>
       <c r="F32" s="162"/>
-      <c r="G32" s="87" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+      <c r="G32" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H32" s="172"/>
-      <c r="I32" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J32" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K32" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I32" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J32" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K32" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L32" s="187"/>
       <c r="M32" s="188"/>
       <c r="N32" s="171"/>
-      <c r="O32" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P32" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O32" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P32" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q32" s="243"/>
       <c r="R32" s="244"/>
@@ -13279,17 +13047,11 @@
       <c r="Z32" s="166"/>
       <c r="AA32" s="168"/>
       <c r="AB32" s="168"/>
-      <c r="AC32" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC32" s="93"/>
       <c r="AD32" s="168"/>
       <c r="AE32" s="176"/>
       <c r="AF32" s="266"/>
-      <c r="AG32" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG32" s="128"/>
       <c r="AH32" s="186"/>
       <c r="AI32" s="173"/>
       <c r="AJ32" s="174"/>
@@ -13325,44 +13087,36 @@
     </row>
     <row r="33" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="94">
-        <f t="shared" si="10"/>
         <v>27</v>
       </c>
       <c r="B33" s="160"/>
-      <c r="C33" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C33" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D33" s="198"/>
       <c r="E33" s="162"/>
       <c r="F33" s="162"/>
-      <c r="G33" s="87" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+      <c r="G33" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H33" s="172"/>
-      <c r="I33" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J33" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K33" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I33" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J33" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K33" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L33" s="187"/>
       <c r="M33" s="188"/>
       <c r="N33" s="171"/>
-      <c r="O33" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P33" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O33" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P33" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q33" s="243"/>
       <c r="R33" s="244"/>
@@ -13376,17 +13130,11 @@
       <c r="Z33" s="166"/>
       <c r="AA33" s="168"/>
       <c r="AB33" s="168"/>
-      <c r="AC33" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC33" s="93"/>
       <c r="AD33" s="168"/>
       <c r="AE33" s="176"/>
       <c r="AF33" s="266"/>
-      <c r="AG33" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG33" s="128"/>
       <c r="AH33" s="186"/>
       <c r="AI33" s="173"/>
       <c r="AJ33" s="174"/>
@@ -13422,44 +13170,36 @@
     </row>
     <row r="34" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="94">
-        <f t="shared" si="10"/>
         <v>28</v>
       </c>
       <c r="B34" s="160"/>
-      <c r="C34" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C34" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D34" s="183"/>
       <c r="E34" s="162"/>
       <c r="F34" s="162"/>
-      <c r="G34" s="87" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+      <c r="G34" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H34" s="172"/>
-      <c r="I34" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J34" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K34" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I34" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J34" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K34" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L34" s="187"/>
       <c r="M34" s="188"/>
       <c r="N34" s="171"/>
-      <c r="O34" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P34" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O34" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P34" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q34" s="243"/>
       <c r="R34" s="244"/>
@@ -13473,17 +13213,11 @@
       <c r="Z34" s="166"/>
       <c r="AA34" s="168"/>
       <c r="AB34" s="168"/>
-      <c r="AC34" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC34" s="93"/>
       <c r="AD34" s="168"/>
       <c r="AE34" s="176"/>
       <c r="AF34" s="267"/>
-      <c r="AG34" s="128" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG34" s="128"/>
       <c r="AH34" s="186"/>
       <c r="AI34" s="173"/>
       <c r="AJ34" s="174"/>
@@ -13519,44 +13253,36 @@
     </row>
     <row r="35" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="94">
-        <f t="shared" si="10"/>
         <v>29</v>
       </c>
       <c r="B35" s="160"/>
-      <c r="C35" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C35" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D35" s="198"/>
       <c r="E35" s="162"/>
       <c r="F35" s="162"/>
-      <c r="G35" s="87" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+      <c r="G35" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H35" s="172"/>
-      <c r="I35" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J35" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K35" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I35" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J35" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K35" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L35" s="187"/>
       <c r="M35" s="188"/>
       <c r="N35" s="171"/>
-      <c r="O35" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P35" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O35" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P35" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q35" s="243"/>
       <c r="R35" s="244"/>
@@ -13570,17 +13296,11 @@
       <c r="Z35" s="166"/>
       <c r="AA35" s="168"/>
       <c r="AB35" s="168"/>
-      <c r="AC35" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC35" s="93"/>
       <c r="AD35" s="168"/>
       <c r="AE35" s="176"/>
       <c r="AF35" s="266"/>
-      <c r="AG35" s="127" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG35" s="127"/>
       <c r="AH35" s="186"/>
       <c r="AI35" s="173"/>
       <c r="AJ35" s="174"/>
@@ -13616,44 +13336,36 @@
     </row>
     <row r="36" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="94">
-        <f t="shared" si="10"/>
         <v>30</v>
       </c>
       <c r="B36" s="160"/>
-      <c r="C36" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C36" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D36" s="183"/>
       <c r="E36" s="162"/>
       <c r="F36" s="162"/>
-      <c r="G36" s="87" t="str">
-        <f t="shared" si="11"/>
-        <v/>
+      <c r="G36" s="87" t="s">
+        <v>106</v>
       </c>
       <c r="H36" s="172"/>
-      <c r="I36" s="88" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J36" s="89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K36" s="88" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I36" s="88" t="s">
+        <v>106</v>
+      </c>
+      <c r="J36" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="K36" s="88" t="s">
+        <v>106</v>
       </c>
       <c r="L36" s="187"/>
       <c r="M36" s="188"/>
       <c r="N36" s="171"/>
-      <c r="O36" s="90" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P36" s="90" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O36" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="P36" s="90" t="s">
+        <v>106</v>
       </c>
       <c r="Q36" s="243"/>
       <c r="R36" s="244"/>
@@ -13667,17 +13379,11 @@
       <c r="Z36" s="166"/>
       <c r="AA36" s="168"/>
       <c r="AB36" s="168"/>
-      <c r="AC36" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC36" s="93"/>
       <c r="AD36" s="168"/>
       <c r="AE36" s="176"/>
       <c r="AF36" s="268"/>
-      <c r="AG36" s="127" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG36" s="127"/>
       <c r="AH36" s="186"/>
       <c r="AI36" s="173"/>
       <c r="AJ36" s="174"/>
@@ -13713,44 +13419,36 @@
     </row>
     <row r="37" spans="1:65" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="95">
-        <f t="shared" si="10"/>
         <v>31</v>
       </c>
       <c r="B37" s="160"/>
-      <c r="C37" s="86" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C37" s="86" t="s">
+        <v>106</v>
       </c>
       <c r="D37" s="198"/>
       <c r="E37" s="162"/>
       <c r="F37" s="162"/>
-      <c r="G37" s="96" t="str">
-        <f t="shared" si="9"/>
-        <v/>
+      <c r="G37" s="96" t="s">
+        <v>106</v>
       </c>
       <c r="H37" s="179"/>
-      <c r="I37" s="97" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J37" s="98" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K37" s="97" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="I37" s="97" t="s">
+        <v>106</v>
+      </c>
+      <c r="J37" s="98" t="s">
+        <v>106</v>
+      </c>
+      <c r="K37" s="97" t="s">
+        <v>106</v>
       </c>
       <c r="L37" s="191"/>
       <c r="M37" s="192"/>
       <c r="N37" s="177"/>
-      <c r="O37" s="99" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="P37" s="99" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="O37" s="99" t="s">
+        <v>106</v>
+      </c>
+      <c r="P37" s="99" t="s">
+        <v>106</v>
       </c>
       <c r="Q37" s="237"/>
       <c r="R37" s="238"/>
@@ -13764,17 +13462,11 @@
       <c r="Z37" s="166"/>
       <c r="AA37" s="168"/>
       <c r="AB37" s="168"/>
-      <c r="AC37" s="93" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC37" s="93"/>
       <c r="AD37" s="168"/>
       <c r="AE37" s="176"/>
       <c r="AF37" s="189"/>
-      <c r="AG37" s="127" t="str">
-        <f t="shared" si="8"/>
-        <v>REDO</v>
-      </c>
+      <c r="AG37" s="127"/>
       <c r="AH37" s="186"/>
       <c r="AI37" s="173"/>
       <c r="AJ37" s="174"/>
@@ -13813,11 +13505,9 @@
         <v>65</v>
       </c>
       <c r="B38" s="101">
-        <f>SUM(B7:B37)</f>
         <v>0</v>
       </c>
       <c r="C38" s="102">
-        <f>SUM(C7:C37)</f>
         <v>0</v>
       </c>
       <c r="D38" s="103"/>
@@ -13825,57 +13515,44 @@
       <c r="F38" s="104"/>
       <c r="G38" s="105"/>
       <c r="H38" s="105">
-        <f t="shared" ref="H38:M38" si="12">SUM(H7:H37)</f>
         <v>0</v>
       </c>
       <c r="I38" s="106">
-        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J38" s="105">
-        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="K38" s="107">
-        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="L38" s="193">
-        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="M38" s="108">
-        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="N38" s="109"/>
       <c r="O38" s="110">
-        <f>SUM(O7:O37)</f>
         <v>0</v>
       </c>
       <c r="P38" s="110">
-        <f>SUM(P7:P37)</f>
         <v>0</v>
       </c>
       <c r="Q38" s="111">
-        <f>SUM(Q7:Q37)</f>
         <v>0</v>
       </c>
       <c r="R38" s="112">
-        <f>SUM(R7:R37)</f>
         <v>0</v>
       </c>
       <c r="S38" s="252"/>
       <c r="T38" s="113">
-        <f>SUM(T7:T37)</f>
         <v>0</v>
       </c>
       <c r="U38" s="114">
-        <f>SUM(U7:U37)</f>
         <v>9</v>
       </c>
       <c r="V38" s="114">
-        <f>SUM(V7:V37)</f>
         <v>0</v>
       </c>
       <c r="W38" s="113"/>
@@ -13884,10 +13561,7 @@
       <c r="Z38" s="113"/>
       <c r="AA38" s="100"/>
       <c r="AB38" s="100"/>
-      <c r="AC38" s="124" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="AC38" s="124"/>
       <c r="AD38" s="100"/>
       <c r="AE38" s="117"/>
       <c r="AF38" s="125"/>
@@ -14007,7 +13681,6 @@
       </c>
       <c r="G40" s="229"/>
       <c r="H40" s="230">
-        <f>+H38*6.2898</f>
         <v>0</v>
       </c>
       <c r="I40" s="38"/>
@@ -14080,10 +13753,7 @@
         <v>68</v>
       </c>
       <c r="G41" s="229"/>
-      <c r="H41" s="230" t="e">
-        <f>+H40/((B38+C38)/24)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="H41" s="230"/>
       <c r="I41" s="38"/>
       <c r="J41" s="38"/>
       <c r="K41" s="38"/>
@@ -14154,10 +13824,7 @@
         <v>70</v>
       </c>
       <c r="G42" s="234"/>
-      <c r="H42" s="235" t="e">
-        <f>+H40/(B38/24)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="H42" s="235"/>
       <c r="I42" s="38"/>
       <c r="J42" s="38"/>
       <c r="K42" s="38"/>
@@ -14292,10 +13959,7 @@
       <c r="D44" s="123" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="236">
-        <f>IF(E41+E42+E43=E40,E40,"Oil, Gas and Sand values do not equal the Initial Tank Gauge. Readjust Values.")</f>
-        <v>0</v>
-      </c>
+      <c r="E44" s="236"/>
       <c r="F44" s="190"/>
       <c r="G44" s="190"/>
       <c r="H44" s="190"/>
@@ -28580,12 +28244,12 @@
       <c r="F1" s="202" t="s">
         <v>80</v>
       </c>
-      <c r="G1" s="297" t="s">
+      <c r="G1" s="304" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="298"/>
-      <c r="I1" s="298"/>
-      <c r="J1" s="298"/>
+      <c r="H1" s="305"/>
+      <c r="I1" s="305"/>
+      <c r="J1" s="305"/>
       <c r="K1" s="291"/>
       <c r="L1" s="203"/>
       <c r="M1" s="129" t="s">
@@ -28607,13 +28271,13 @@
         <v>86</v>
       </c>
       <c r="S1" s="203"/>
-      <c r="T1" s="302" t="s">
+      <c r="T1" s="300" t="s">
         <v>104</v>
       </c>
-      <c r="U1" s="302"/>
-      <c r="V1" s="302"/>
+      <c r="U1" s="300"/>
+      <c r="V1" s="300"/>
       <c r="W1" s="1"/>
-      <c r="X1" s="299" t="s">
+      <c r="X1" s="301" t="s">
         <v>87</v>
       </c>
       <c r="Y1" s="287"/>
@@ -28682,11 +28346,11 @@
       <c r="D3" s="129"/>
       <c r="E3" s="215"/>
       <c r="F3" s="215"/>
-      <c r="G3" s="294"/>
-      <c r="H3" s="300"/>
-      <c r="I3" s="300"/>
-      <c r="J3" s="300"/>
-      <c r="K3" s="301"/>
+      <c r="G3" s="297"/>
+      <c r="H3" s="302"/>
+      <c r="I3" s="302"/>
+      <c r="J3" s="302"/>
+      <c r="K3" s="303"/>
       <c r="L3" s="203"/>
       <c r="M3" s="203">
         <v>1</v>
@@ -28724,11 +28388,11 @@
       <c r="D4" s="129"/>
       <c r="E4" s="215"/>
       <c r="F4" s="215"/>
-      <c r="G4" s="294"/>
-      <c r="H4" s="300"/>
-      <c r="I4" s="300"/>
-      <c r="J4" s="300"/>
-      <c r="K4" s="301"/>
+      <c r="G4" s="297"/>
+      <c r="H4" s="302"/>
+      <c r="I4" s="302"/>
+      <c r="J4" s="302"/>
+      <c r="K4" s="303"/>
       <c r="L4" s="203"/>
       <c r="M4" s="203">
         <v>2</v>
@@ -28766,11 +28430,11 @@
       <c r="D5" s="217"/>
       <c r="E5" s="215"/>
       <c r="F5" s="215"/>
-      <c r="G5" s="294"/>
-      <c r="H5" s="300"/>
-      <c r="I5" s="300"/>
-      <c r="J5" s="300"/>
-      <c r="K5" s="301"/>
+      <c r="G5" s="297"/>
+      <c r="H5" s="302"/>
+      <c r="I5" s="302"/>
+      <c r="J5" s="302"/>
+      <c r="K5" s="303"/>
       <c r="L5" s="203"/>
       <c r="M5" s="203">
         <v>3</v>
@@ -28808,11 +28472,11 @@
       <c r="D6" s="260"/>
       <c r="E6" s="215"/>
       <c r="F6" s="215"/>
-      <c r="G6" s="294"/>
-      <c r="H6" s="300"/>
-      <c r="I6" s="300"/>
-      <c r="J6" s="300"/>
-      <c r="K6" s="301"/>
+      <c r="G6" s="297"/>
+      <c r="H6" s="302"/>
+      <c r="I6" s="302"/>
+      <c r="J6" s="302"/>
+      <c r="K6" s="303"/>
       <c r="L6" s="203"/>
       <c r="M6" s="203">
         <v>4</v>
@@ -28850,11 +28514,11 @@
       <c r="D7" s="217"/>
       <c r="E7" s="215"/>
       <c r="F7" s="215"/>
-      <c r="G7" s="294"/>
-      <c r="H7" s="300"/>
-      <c r="I7" s="300"/>
-      <c r="J7" s="300"/>
-      <c r="K7" s="301"/>
+      <c r="G7" s="297"/>
+      <c r="H7" s="302"/>
+      <c r="I7" s="302"/>
+      <c r="J7" s="302"/>
+      <c r="K7" s="303"/>
       <c r="L7" s="203"/>
       <c r="M7" s="203">
         <v>5</v>
@@ -28892,11 +28556,11 @@
       <c r="D8" s="217"/>
       <c r="E8" s="215"/>
       <c r="F8" s="215"/>
-      <c r="G8" s="294"/>
-      <c r="H8" s="300"/>
-      <c r="I8" s="300"/>
-      <c r="J8" s="300"/>
-      <c r="K8" s="301"/>
+      <c r="G8" s="297"/>
+      <c r="H8" s="302"/>
+      <c r="I8" s="302"/>
+      <c r="J8" s="302"/>
+      <c r="K8" s="303"/>
       <c r="L8" s="203"/>
       <c r="M8" s="203">
         <v>6</v>
@@ -28934,11 +28598,11 @@
       <c r="D9" s="217"/>
       <c r="E9" s="215"/>
       <c r="F9" s="215"/>
-      <c r="G9" s="294"/>
-      <c r="H9" s="300"/>
-      <c r="I9" s="300"/>
-      <c r="J9" s="300"/>
-      <c r="K9" s="301"/>
+      <c r="G9" s="297"/>
+      <c r="H9" s="302"/>
+      <c r="I9" s="302"/>
+      <c r="J9" s="302"/>
+      <c r="K9" s="303"/>
       <c r="L9" s="203"/>
       <c r="M9" s="203">
         <v>7</v>
@@ -28976,11 +28640,11 @@
       <c r="D10" s="217"/>
       <c r="E10" s="215"/>
       <c r="F10" s="215"/>
-      <c r="G10" s="294"/>
-      <c r="H10" s="295"/>
-      <c r="I10" s="295"/>
-      <c r="J10" s="295"/>
-      <c r="K10" s="296"/>
+      <c r="G10" s="297"/>
+      <c r="H10" s="298"/>
+      <c r="I10" s="298"/>
+      <c r="J10" s="298"/>
+      <c r="K10" s="299"/>
       <c r="L10" s="203"/>
       <c r="M10" s="203">
         <v>8</v>
@@ -29018,11 +28682,11 @@
       <c r="D11" s="129"/>
       <c r="E11" s="215"/>
       <c r="F11" s="215"/>
-      <c r="G11" s="294"/>
-      <c r="H11" s="295"/>
-      <c r="I11" s="295"/>
-      <c r="J11" s="295"/>
-      <c r="K11" s="296"/>
+      <c r="G11" s="297"/>
+      <c r="H11" s="298"/>
+      <c r="I11" s="298"/>
+      <c r="J11" s="298"/>
+      <c r="K11" s="299"/>
       <c r="L11" s="203"/>
       <c r="M11" s="203">
         <v>9</v>
@@ -29060,11 +28724,11 @@
       <c r="D12" s="217"/>
       <c r="E12" s="157"/>
       <c r="F12" s="215"/>
-      <c r="G12" s="294"/>
-      <c r="H12" s="295"/>
-      <c r="I12" s="295"/>
-      <c r="J12" s="295"/>
-      <c r="K12" s="296"/>
+      <c r="G12" s="297"/>
+      <c r="H12" s="298"/>
+      <c r="I12" s="298"/>
+      <c r="J12" s="298"/>
+      <c r="K12" s="299"/>
       <c r="L12" s="203"/>
       <c r="M12" s="203">
         <v>10</v>
@@ -29102,11 +28766,11 @@
       <c r="D13" s="129"/>
       <c r="E13" s="215"/>
       <c r="F13" s="215"/>
-      <c r="G13" s="294"/>
-      <c r="H13" s="295"/>
-      <c r="I13" s="295"/>
-      <c r="J13" s="295"/>
-      <c r="K13" s="296"/>
+      <c r="G13" s="297"/>
+      <c r="H13" s="298"/>
+      <c r="I13" s="298"/>
+      <c r="J13" s="298"/>
+      <c r="K13" s="299"/>
       <c r="L13" s="203"/>
       <c r="M13" s="203">
         <v>11</v>
@@ -29144,11 +28808,11 @@
       <c r="D14" s="217"/>
       <c r="E14" s="215"/>
       <c r="F14" s="215"/>
-      <c r="G14" s="294"/>
-      <c r="H14" s="295"/>
-      <c r="I14" s="295"/>
-      <c r="J14" s="295"/>
-      <c r="K14" s="296"/>
+      <c r="G14" s="297"/>
+      <c r="H14" s="298"/>
+      <c r="I14" s="298"/>
+      <c r="J14" s="298"/>
+      <c r="K14" s="299"/>
       <c r="L14" s="203"/>
       <c r="M14" s="203">
         <v>12</v>
@@ -29186,11 +28850,11 @@
       <c r="D15" s="129"/>
       <c r="E15" s="157"/>
       <c r="F15" s="215"/>
-      <c r="G15" s="294"/>
-      <c r="H15" s="295"/>
-      <c r="I15" s="295"/>
-      <c r="J15" s="295"/>
-      <c r="K15" s="296"/>
+      <c r="G15" s="297"/>
+      <c r="H15" s="298"/>
+      <c r="I15" s="298"/>
+      <c r="J15" s="298"/>
+      <c r="K15" s="299"/>
       <c r="L15" s="203"/>
       <c r="M15" s="203">
         <v>13</v>
@@ -29228,11 +28892,11 @@
       <c r="D16" s="129"/>
       <c r="E16" s="157"/>
       <c r="F16" s="215"/>
-      <c r="G16" s="294"/>
-      <c r="H16" s="295"/>
-      <c r="I16" s="295"/>
-      <c r="J16" s="295"/>
-      <c r="K16" s="296"/>
+      <c r="G16" s="297"/>
+      <c r="H16" s="298"/>
+      <c r="I16" s="298"/>
+      <c r="J16" s="298"/>
+      <c r="K16" s="299"/>
       <c r="L16" s="203"/>
       <c r="M16" s="203">
         <v>14</v>
@@ -29270,11 +28934,11 @@
       <c r="D17" s="129"/>
       <c r="E17" s="157"/>
       <c r="F17" s="215"/>
-      <c r="G17" s="294"/>
-      <c r="H17" s="295"/>
-      <c r="I17" s="295"/>
-      <c r="J17" s="295"/>
-      <c r="K17" s="296"/>
+      <c r="G17" s="297"/>
+      <c r="H17" s="298"/>
+      <c r="I17" s="298"/>
+      <c r="J17" s="298"/>
+      <c r="K17" s="299"/>
       <c r="L17" s="203"/>
       <c r="M17" s="203">
         <v>15</v>
@@ -29312,11 +28976,11 @@
       <c r="D18" s="129"/>
       <c r="E18" s="157"/>
       <c r="F18" s="215"/>
-      <c r="G18" s="294"/>
-      <c r="H18" s="295"/>
-      <c r="I18" s="295"/>
-      <c r="J18" s="295"/>
-      <c r="K18" s="296"/>
+      <c r="G18" s="297"/>
+      <c r="H18" s="298"/>
+      <c r="I18" s="298"/>
+      <c r="J18" s="298"/>
+      <c r="K18" s="299"/>
       <c r="L18" s="203"/>
       <c r="M18" s="203">
         <v>16</v>
@@ -29354,11 +29018,11 @@
       <c r="D19" s="129"/>
       <c r="E19" s="215"/>
       <c r="F19" s="215"/>
-      <c r="G19" s="294"/>
-      <c r="H19" s="295"/>
-      <c r="I19" s="295"/>
-      <c r="J19" s="295"/>
-      <c r="K19" s="296"/>
+      <c r="G19" s="297"/>
+      <c r="H19" s="298"/>
+      <c r="I19" s="298"/>
+      <c r="J19" s="298"/>
+      <c r="K19" s="299"/>
       <c r="L19" s="203"/>
       <c r="M19" s="203">
         <v>17</v>
@@ -29396,11 +29060,11 @@
       <c r="D20" s="217"/>
       <c r="E20" s="215"/>
       <c r="F20" s="215"/>
-      <c r="G20" s="294"/>
-      <c r="H20" s="295"/>
-      <c r="I20" s="295"/>
-      <c r="J20" s="295"/>
-      <c r="K20" s="296"/>
+      <c r="G20" s="297"/>
+      <c r="H20" s="298"/>
+      <c r="I20" s="298"/>
+      <c r="J20" s="298"/>
+      <c r="K20" s="299"/>
       <c r="L20" s="203"/>
       <c r="M20" s="203">
         <v>18</v>
@@ -29438,11 +29102,11 @@
       <c r="D21" s="217"/>
       <c r="E21" s="215"/>
       <c r="F21" s="215"/>
-      <c r="G21" s="294"/>
-      <c r="H21" s="295"/>
-      <c r="I21" s="295"/>
-      <c r="J21" s="295"/>
-      <c r="K21" s="296"/>
+      <c r="G21" s="297"/>
+      <c r="H21" s="298"/>
+      <c r="I21" s="298"/>
+      <c r="J21" s="298"/>
+      <c r="K21" s="299"/>
       <c r="L21" s="203"/>
       <c r="M21" s="203">
         <v>19</v>
@@ -29480,11 +29144,11 @@
       <c r="D22" s="129"/>
       <c r="E22" s="157"/>
       <c r="F22" s="215"/>
-      <c r="G22" s="294"/>
-      <c r="H22" s="295"/>
-      <c r="I22" s="295"/>
-      <c r="J22" s="295"/>
-      <c r="K22" s="296"/>
+      <c r="G22" s="297"/>
+      <c r="H22" s="298"/>
+      <c r="I22" s="298"/>
+      <c r="J22" s="298"/>
+      <c r="K22" s="299"/>
       <c r="L22" s="203"/>
       <c r="M22" s="203">
         <v>20</v>
@@ -29522,11 +29186,11 @@
       <c r="D23" s="217"/>
       <c r="E23" s="215"/>
       <c r="F23" s="215"/>
-      <c r="G23" s="294"/>
-      <c r="H23" s="295"/>
-      <c r="I23" s="295"/>
-      <c r="J23" s="295"/>
-      <c r="K23" s="296"/>
+      <c r="G23" s="297"/>
+      <c r="H23" s="298"/>
+      <c r="I23" s="298"/>
+      <c r="J23" s="298"/>
+      <c r="K23" s="299"/>
       <c r="L23" s="203"/>
       <c r="M23" s="203">
         <v>21</v>
@@ -29606,11 +29270,11 @@
       <c r="D25" s="217"/>
       <c r="E25" s="157"/>
       <c r="F25" s="215"/>
-      <c r="G25" s="294"/>
-      <c r="H25" s="295"/>
-      <c r="I25" s="295"/>
-      <c r="J25" s="295"/>
-      <c r="K25" s="296"/>
+      <c r="G25" s="297"/>
+      <c r="H25" s="298"/>
+      <c r="I25" s="298"/>
+      <c r="J25" s="298"/>
+      <c r="K25" s="299"/>
       <c r="L25" s="203"/>
       <c r="M25" s="203">
         <v>23</v>
@@ -29648,11 +29312,11 @@
       <c r="D26" s="217"/>
       <c r="E26" s="129"/>
       <c r="F26" s="215"/>
-      <c r="G26" s="294"/>
-      <c r="H26" s="295"/>
-      <c r="I26" s="295"/>
-      <c r="J26" s="295"/>
-      <c r="K26" s="296"/>
+      <c r="G26" s="297"/>
+      <c r="H26" s="298"/>
+      <c r="I26" s="298"/>
+      <c r="J26" s="298"/>
+      <c r="K26" s="299"/>
       <c r="L26" s="203"/>
       <c r="M26" s="203">
         <v>24</v>
@@ -29690,11 +29354,11 @@
       <c r="D27" s="217"/>
       <c r="E27" s="157"/>
       <c r="F27" s="215"/>
-      <c r="G27" s="294"/>
-      <c r="H27" s="295"/>
-      <c r="I27" s="295"/>
-      <c r="J27" s="295"/>
-      <c r="K27" s="296"/>
+      <c r="G27" s="297"/>
+      <c r="H27" s="298"/>
+      <c r="I27" s="298"/>
+      <c r="J27" s="298"/>
+      <c r="K27" s="299"/>
       <c r="L27" s="203"/>
       <c r="M27" s="203">
         <v>25</v>
@@ -29732,11 +29396,11 @@
       <c r="D28" s="129"/>
       <c r="E28" s="157"/>
       <c r="F28" s="215"/>
-      <c r="G28" s="294"/>
-      <c r="H28" s="295"/>
-      <c r="I28" s="295"/>
-      <c r="J28" s="295"/>
-      <c r="K28" s="296"/>
+      <c r="G28" s="297"/>
+      <c r="H28" s="298"/>
+      <c r="I28" s="298"/>
+      <c r="J28" s="298"/>
+      <c r="K28" s="299"/>
       <c r="L28" s="203"/>
       <c r="M28" s="203">
         <v>26</v>
@@ -29774,11 +29438,11 @@
       <c r="D29" s="129"/>
       <c r="E29" s="215"/>
       <c r="F29" s="215"/>
-      <c r="G29" s="294"/>
-      <c r="H29" s="295"/>
-      <c r="I29" s="295"/>
-      <c r="J29" s="295"/>
-      <c r="K29" s="296"/>
+      <c r="G29" s="297"/>
+      <c r="H29" s="298"/>
+      <c r="I29" s="298"/>
+      <c r="J29" s="298"/>
+      <c r="K29" s="299"/>
       <c r="L29" s="203"/>
       <c r="M29" s="203">
         <v>27</v>
@@ -29816,11 +29480,11 @@
       <c r="D30" s="217"/>
       <c r="E30" s="215"/>
       <c r="F30" s="215"/>
-      <c r="G30" s="294"/>
-      <c r="H30" s="295"/>
-      <c r="I30" s="295"/>
-      <c r="J30" s="295"/>
-      <c r="K30" s="296"/>
+      <c r="G30" s="297"/>
+      <c r="H30" s="298"/>
+      <c r="I30" s="298"/>
+      <c r="J30" s="298"/>
+      <c r="K30" s="299"/>
       <c r="L30" s="203"/>
       <c r="M30" s="203">
         <v>28</v>
@@ -29858,11 +29522,11 @@
       <c r="D31" s="217"/>
       <c r="E31" s="157"/>
       <c r="F31" s="215"/>
-      <c r="G31" s="294"/>
-      <c r="H31" s="295"/>
-      <c r="I31" s="295"/>
-      <c r="J31" s="295"/>
-      <c r="K31" s="296"/>
+      <c r="G31" s="297"/>
+      <c r="H31" s="298"/>
+      <c r="I31" s="298"/>
+      <c r="J31" s="298"/>
+      <c r="K31" s="299"/>
       <c r="L31" s="203"/>
       <c r="M31" s="203">
         <v>29</v>
@@ -29900,11 +29564,11 @@
       <c r="D32" s="129"/>
       <c r="E32" s="215"/>
       <c r="F32" s="215"/>
-      <c r="G32" s="294"/>
-      <c r="H32" s="295"/>
-      <c r="I32" s="295"/>
-      <c r="J32" s="295"/>
-      <c r="K32" s="296"/>
+      <c r="G32" s="297"/>
+      <c r="H32" s="298"/>
+      <c r="I32" s="298"/>
+      <c r="J32" s="298"/>
+      <c r="K32" s="299"/>
       <c r="L32" s="203"/>
       <c r="M32" s="203">
         <v>30</v>
@@ -29942,11 +29606,11 @@
       <c r="D33" s="203"/>
       <c r="E33" s="157"/>
       <c r="F33" s="215"/>
-      <c r="G33" s="294"/>
-      <c r="H33" s="295"/>
-      <c r="I33" s="295"/>
-      <c r="J33" s="295"/>
-      <c r="K33" s="296"/>
+      <c r="G33" s="297"/>
+      <c r="H33" s="298"/>
+      <c r="I33" s="298"/>
+      <c r="J33" s="298"/>
+      <c r="K33" s="299"/>
       <c r="L33" s="203"/>
       <c r="M33" s="203">
         <v>31</v>
@@ -29982,11 +29646,11 @@
       <c r="D34" s="129"/>
       <c r="E34" s="129"/>
       <c r="F34" s="215"/>
-      <c r="G34" s="294"/>
-      <c r="H34" s="295"/>
-      <c r="I34" s="295"/>
-      <c r="J34" s="295"/>
-      <c r="K34" s="296"/>
+      <c r="G34" s="297"/>
+      <c r="H34" s="298"/>
+      <c r="I34" s="298"/>
+      <c r="J34" s="298"/>
+      <c r="K34" s="299"/>
       <c r="L34" s="203"/>
       <c r="M34" s="203"/>
       <c r="N34" s="203"/>
@@ -30038,11 +29702,11 @@
       <c r="D35" s="129"/>
       <c r="E35" s="157"/>
       <c r="F35" s="215"/>
-      <c r="G35" s="294"/>
-      <c r="H35" s="295"/>
-      <c r="I35" s="295"/>
-      <c r="J35" s="295"/>
-      <c r="K35" s="296"/>
+      <c r="G35" s="297"/>
+      <c r="H35" s="298"/>
+      <c r="I35" s="298"/>
+      <c r="J35" s="298"/>
+      <c r="K35" s="299"/>
       <c r="L35" s="203"/>
       <c r="M35" s="203"/>
       <c r="N35" s="220">
@@ -30080,11 +29744,11 @@
       <c r="D36" s="222"/>
       <c r="E36" s="222"/>
       <c r="F36" s="223"/>
-      <c r="G36" s="303"/>
-      <c r="H36" s="304"/>
-      <c r="I36" s="304"/>
-      <c r="J36" s="304"/>
-      <c r="K36" s="305"/>
+      <c r="G36" s="294"/>
+      <c r="H36" s="295"/>
+      <c r="I36" s="295"/>
+      <c r="J36" s="295"/>
+      <c r="K36" s="296"/>
       <c r="L36" s="203"/>
       <c r="M36" s="203"/>
       <c r="N36" s="203"/>
@@ -37271,18 +36935,16 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="X1:AA1"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="G1:K1"/>
     <mergeCell ref="G10:K10"/>
     <mergeCell ref="G23:K23"/>
     <mergeCell ref="G12:K12"/>
@@ -37297,16 +36959,18 @@
     <mergeCell ref="G20:K20"/>
     <mergeCell ref="G21:K21"/>
     <mergeCell ref="G22:K22"/>
-    <mergeCell ref="T1:V1"/>
-    <mergeCell ref="X1:AA1"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G9:K9"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="decimal" operator="lessThan" allowBlank="1" showInputMessage="1" prompt="INPUT TICKET NUMBER - Please input the ticket number. Use &quot;/&quot; to separate multiple ticket numbers." sqref="AB22:AB28 X3:AA33 C22:C28 AB9:AB17 C9:C17" xr:uid="{6EBA5DD2-9520-1C44-B6DD-78BB8475944E}">
@@ -37387,7 +37051,7 @@
         <v>#REF!</v>
       </c>
       <c r="N3" s="132" t="str">
-        <f ca="1">'Well Template'!AE1</f>
+        <f>'Well Template'!AE1</f>
         <v>Well Template</v>
       </c>
       <c r="O3" s="132" t="e">
@@ -41018,7 +40682,7 @@
         <v>#REF!</v>
       </c>
       <c r="N38" s="132" t="str">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>Well Template</v>
       </c>
       <c r="O38" s="132" t="e">
@@ -44650,7 +44314,7 @@
         <v>#REF!</v>
       </c>
       <c r="N74" s="132" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>Well Template</v>
       </c>
       <c r="O74" s="132" t="e">
@@ -48811,7 +48475,7 @@
         <v>#REF!</v>
       </c>
       <c r="N111" s="132" t="str">
-        <f t="shared" ca="1" si="11"/>
+        <f t="shared" si="11"/>
         <v>Well Template</v>
       </c>
       <c r="O111" s="132" t="e">
@@ -52459,7 +52123,7 @@
         <v>#REF!</v>
       </c>
       <c r="N147" s="132" t="str">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" si="15"/>
         <v>Well Template</v>
       </c>
       <c r="O147" s="132" t="e">
@@ -56093,7 +55757,7 @@
         <v>#REF!</v>
       </c>
       <c r="N183" s="132" t="str">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" si="20"/>
         <v>Well Template</v>
       </c>
       <c r="O183" s="132" t="e">

</xml_diff>